<commit_message>
Corrected Reserves.xlsx input file for 2020 Refined; Iron values off by 1000.
</commit_message>
<xml_diff>
--- a/Data point Supporting files/Germany 2020/Reserves.xlsx
+++ b/Data point Supporting files/Germany 2020/Reserves.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="23"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Aluminium" sheetId="1" state="visible" r:id="rId2"/>
@@ -841,10 +841,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.06"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -860,7 +861,7 @@
         <v>13</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>3000000</v>
+        <v>3000000000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -868,7 +869,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>50000000</v>
+        <v>50000000000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -876,7 +877,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>34000000</v>
+        <v>34000000000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -884,7 +885,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>6000000</v>
+        <v>6000000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -892,7 +893,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>20000000</v>
+        <v>20000000000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -900,7 +901,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>5500000</v>
+        <v>5500000000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -908,7 +909,7 @@
         <v>46</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>2700000</v>
+        <v>2700000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -916,7 +917,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>2500000</v>
+        <v>2500000000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -924,7 +925,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>25000000</v>
+        <v>25000000000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -932,7 +933,7 @@
         <v>27</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>1000000</v>
+        <v>1000000000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -940,7 +941,7 @@
         <v>47</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>1300000</v>
+        <v>1300000000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -948,7 +949,7 @@
         <v>48</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>6500000</v>
+        <v>6500000000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -956,7 +957,7 @@
         <v>15</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>18000000</v>
+        <v>18000000000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -964,7 +965,7 @@
         <v>16</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>180000000</v>
+        <v>180000000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>